<commit_message>
Phase 4: pre-step architecture; ADSL structurally correct
</commit_message>
<xml_diff>
--- a/adam_spec.xlsx
+++ b/adam_spec.xlsx
@@ -509,19 +509,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="70" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="58" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -572,6 +573,11 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Derivation</t>
         </is>
       </c>
@@ -612,6 +618,11 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
           <t>DM.STUDYID</t>
         </is>
       </c>
@@ -652,6 +663,11 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
           <t>DM.USUBJID</t>
         </is>
       </c>
@@ -692,6 +708,11 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
           <t>DM.SUBJID</t>
         </is>
       </c>
@@ -732,6 +753,11 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
           <t>DM.SITEID</t>
         </is>
       </c>
@@ -772,6 +798,11 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
           <t>DM.AGE</t>
         </is>
       </c>
@@ -816,6 +847,11 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
           <t>DM.AGEU</t>
         </is>
       </c>
@@ -859,6 +895,11 @@
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>If AGE &lt; 65 then AGEGR1 = "&lt;65"; else if 65 &lt;= AGE &lt;= 80 then AGEGR1 = "65-80"; else if AGE &gt; 80 then AGEGR1 = "&gt;80".</t>
         </is>
@@ -900,6 +941,11 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
           <t>Numeric code for AGEGR1: "&lt;65"=1; "65-80"=2; "&gt;80"=3.</t>
         </is>
       </c>
@@ -944,6 +990,11 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
           <t>DM.SEX</t>
         </is>
       </c>
@@ -987,6 +1038,11 @@
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>DM.RACE</t>
         </is>
@@ -1028,6 +1084,11 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
           <t>DM.ARM</t>
         </is>
       </c>
@@ -1071,6 +1132,11 @@
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Set to DM.ARM.</t>
         </is>
@@ -1112,6 +1178,11 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
           <t>Numeric code for TRT01P: "Placebo"=0; "Drug A 50mg"=1; "Drug A 100mg"=2.</t>
         </is>
       </c>
@@ -1156,7 +1227,12 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Set to EX.EXTRT of the first exposure record. If subject never dosed, set to TRT01P.</t>
+          <t>EX_SUMMARY</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>EX.EXTRT of the first exposure record (min EXSTDTC) where EXDOSE &gt; 0. If subject never dosed, set to TRT01P.</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1276,12 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Date part of the earliest non-missing EX.EXSTDTC where EX.EXDOSE &gt; 0. Numeric SAS date.</t>
+          <t>EX_SUMMARY</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Date part of the earliest non-missing EX.EXSTDTC where EX.EXDOSE &gt; 0.</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1325,12 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Date part of the latest non-missing EX.EXENDTC where EX.EXDOSE &gt; 0. Numeric SAS date.</t>
+          <t>EX_SUMMARY</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Date part of the latest non-missing EX.EXENDTC where EX.EXDOSE &gt; 0.</t>
         </is>
       </c>
     </row>
@@ -1284,6 +1370,11 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
           <t>TRTEDT - TRTSDT + 1. Missing if either date is missing.</t>
         </is>
       </c>
@@ -1328,7 +1419,12 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Y if subject has at least one non-missing TRTSDT; else N.</t>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Y if TRTSDT is non-missing; else N.</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1468,12 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Y if subject is randomised (DM.ARM is not missing and not "Screen Failure"); else N.</t>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Y if ARM is not missing and not "Screen Failure"; else N.</t>
         </is>
       </c>
     </row>
@@ -1415,6 +1516,11 @@
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>DM.DTHFL</t>
         </is>

</xml_diff>

<commit_message>
Phase 4: SUPPDM transpose pre-step; prompt rule for transposed qualifiers
</commit_message>
<xml_diff>
--- a/adam_spec.xlsx
+++ b/adam_spec.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datasets" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variables" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codelists" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SuppQualifiers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codelists" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -509,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1059,12 +1060,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>RACEOTH</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Description of Planned Arm</t>
+          <t>Race, Other Specify</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1073,7 +1074,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr"/>
@@ -1084,12 +1085,12 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>DM</t>
+          <t>SUPPDM</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>DM.ARM</t>
+          <t>SUPPDM QNAM=RACEOTH (QVAL).</t>
         </is>
       </c>
     </row>
@@ -1104,12 +1105,12 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>TRT01P</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Planned Treatment for Period 01</t>
+          <t>Description of Planned Arm</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1121,14 +1122,10 @@
         <v>40</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>TRTP</t>
-        </is>
-      </c>
+      <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Predecessor</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1138,7 +1135,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Set to DM.ARM.</t>
+          <t>DM.ARM</t>
         </is>
       </c>
     </row>
@@ -1153,24 +1150,28 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>TRT01PN</t>
+          <t>TRT01P</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Planned Treatment for Period 01 (N)</t>
+          <t>Planned Treatment for Period 01</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>TRTP</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Derived</t>
@@ -1178,12 +1179,12 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>DERIVED</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Numeric code for TRT01P: "Placebo"=0; "Drug A 50mg"=1; "Drug A 100mg"=2.</t>
+          <t>Set to DM.ARM.</t>
         </is>
       </c>
     </row>
@@ -1198,28 +1199,24 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>TRT01A</t>
+          <t>TRT01PN</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Actual Treatment for Period 01</t>
+          <t>Planned Treatment for Period 01 (N)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>TRTA</t>
-        </is>
-      </c>
+      <c r="H15" s="2" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Derived</t>
@@ -1227,12 +1224,12 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>EX_SUMMARY</t>
+          <t>DERIVED</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>EX.EXTRT of the first exposure record (min EXSTDTC) where EXDOSE &gt; 0. If subject never dosed, set to TRT01P.</t>
+          <t>Numeric code for TRT01P: "Placebo"=0; "Drug A 50mg"=1; "Drug A 100mg"=2.</t>
         </is>
       </c>
     </row>
@@ -1247,28 +1244,28 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>TRTSDT</t>
+          <t>TRT01A</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Date of First Exposure to Treatment</t>
+          <t>Actual Treatment for Period 01</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>DATE9.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>TRTA</t>
+        </is>
+      </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Derived</t>
@@ -1281,7 +1278,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Date part of the earliest non-missing EX.EXSTDTC where EX.EXDOSE &gt; 0.</t>
+          <t>EX.EXTRT of the first exposure record (min EXSTDTC) where EXDOSE &gt; 0. If subject never dosed, set to TRT01P.</t>
         </is>
       </c>
     </row>
@@ -1296,12 +1293,12 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>TRTEDT</t>
+          <t>TRTSDT</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Date of Last Exposure to Treatment</t>
+          <t>Date of First Exposure to Treatment</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1330,7 +1327,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Date part of the latest non-missing EX.EXENDTC where EX.EXDOSE &gt; 0.</t>
+          <t>Date part of the earliest non-missing EX.EXSTDTC where EX.EXDOSE &gt; 0.</t>
         </is>
       </c>
     </row>
@@ -1345,12 +1342,12 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>TRTDURD</t>
+          <t>TRTEDT</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Total Treatment Duration (Days)</t>
+          <t>Date of Last Exposure to Treatment</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1361,7 +1358,11 @@
       <c r="F18" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="G18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>DATE9.</t>
+        </is>
+      </c>
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
@@ -1370,12 +1371,12 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>DERIVED</t>
+          <t>EX_SUMMARY</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>TRTEDT - TRTSDT + 1. Missing if either date is missing.</t>
+          <t>Date part of the latest non-missing EX.EXENDTC where EX.EXDOSE &gt; 0.</t>
         </is>
       </c>
     </row>
@@ -1390,28 +1391,24 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>SAFFL</t>
+          <t>TRTDURD</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Safety Population Flag</t>
+          <t>Total Treatment Duration (Days)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
+      <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr">
         <is>
           <t>Derived</t>
@@ -1424,7 +1421,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Y if TRTSDT is non-missing; else N.</t>
+          <t>TRTEDT - TRTSDT + 1. Missing if either date is missing.</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1436,12 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>ITTFL</t>
+          <t>COMPFL</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Intent-To-Treat Population Flag</t>
+          <t>Study Completion Flag</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1468,12 +1465,12 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>DM</t>
+          <t>DERIVED</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Y if ARM is not missing and not "Screen Failure"; else N.</t>
+          <t>Y if SUPPDM QNAM=COMPLT has QVAL of "Y"; else N.</t>
         </is>
       </c>
     </row>
@@ -1488,12 +1485,12 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>DTHFL</t>
+          <t>SAFFL</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Subject Death Flag</t>
+          <t>Safety Population Flag</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1512,15 +1509,113 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Y if TRTSDT is non-missing; else N.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>ITTFL</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Intent-To-Treat Population Flag</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Y if ARM is not missing and not "Screen Failure"; else N.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>DTHFL</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Subject Death Flag</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
           <t>Predecessor</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>DM.DTHFL</t>
         </is>
@@ -1532,6 +1627,104 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>QNAM</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>QLABEL</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Length</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SUPPDM</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>RACEOTH</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Race, Other Specify</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SUPPDM</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>COMPLT</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Completed Study</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Phase 4: SE epoch pre-step; three domain patterns complete
</commit_message>
<xml_diff>
--- a/adam_spec.xlsx
+++ b/adam_spec.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1436,28 +1436,28 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>COMPFL</t>
+          <t>TRTEPSDT</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Study Completion Flag</t>
+          <t>Treatment Epoch Start Date</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>DATE9.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr">
         <is>
           <t>Derived</t>
@@ -1465,12 +1465,12 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>DERIVED</t>
+          <t>SE_EPOCH</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Y if SUPPDM QNAM=COMPLT has QVAL of "Y"; else N.</t>
+          <t>Date part of SE.SESTDTC for the element where ETCD = "TRT".</t>
         </is>
       </c>
     </row>
@@ -1485,28 +1485,28 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>SAFFL</t>
+          <t>TRTEPEDT</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Safety Population Flag</t>
+          <t>Treatment Epoch End Date</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>DATE9.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr">
         <is>
           <t>Derived</t>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>DERIVED</t>
+          <t>SE_EPOCH</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Y if TRTSDT is non-missing; else N.</t>
+          <t>Date part of SE.SEENDTC for the element where ETCD = "TRT".</t>
         </is>
       </c>
     </row>
@@ -1534,12 +1534,12 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>ITTFL</t>
+          <t>EPOCHFL</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Intent-To-Treat Population Flag</t>
+          <t>Entered Treatment Epoch Flag</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1563,12 +1563,12 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>DM</t>
+          <t>DERIVED</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Y if ARM is not missing and not "Screen Failure"; else N.</t>
+          <t>Y if TRTEPSDT is non-missing; else N.</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1583,12 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>DTHFL</t>
+          <t>COMPFL</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Subject Death Flag</t>
+          <t>Study Completion Flag</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1607,15 +1607,162 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Y if SUPPDM QNAM=COMPLT has QVAL of "Y"; else N.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>SAFFL</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Safety Population Flag</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Y if TRTSDT is non-missing; else N.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>ITTFL</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Intent-To-Treat Population Flag</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Y if ARM is not missing and not "Screen Failure"; else N.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>DTHFL</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Subject Death Flag</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
           <t>Predecessor</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>DM.DTHFL</t>
         </is>

</xml_diff>